<commit_message>
Fix: booking autodetect swept up stale prior-day BKG+PD files
- _autodetect() now scopes to today's upload batch (same mtime date as
  the newest file in the folder) before collecting bkg-role candidates,
  so a leftover 9-10/9-11/9-14-BKG+PD.xls doesn't get combined in
- support multiple booking files properly (load_booking_all, --bkg
  repeatable): today's export split into *PENDING*.xlsx (backlog,
  every TRAN DT before today) + *BKG-3WK*.xls (today + next ~3 weeks) -
  the WK2ND section was silently empty before this since only the
  backlog file was ever detected
- cross-checked combined WK2 totals against the raw files directly

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/HAL Stock HQ - Daily 2026-09-15.xlsx
+++ b/HAL Stock HQ - Daily 2026-09-15.xlsx
@@ -22,7 +22,7 @@
     <numFmt numFmtId="165" formatCode="0;-0;;@"/>
     <numFmt numFmtId="166" formatCode="d/m/yyyy"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="27">
     <font>
       <name val="Tahoma"/>
       <family val="2"/>
@@ -162,6 +162,18 @@
     </font>
     <font>
       <name val="Aptos"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <color rgb="FF0000FF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <b val="1"/>
       <color rgb="FF0000FF"/>
       <sz val="10"/>
     </font>
@@ -171,8 +183,14 @@
       <color rgb="FF0000FF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFFF0000"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -225,6 +243,11 @@
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.7999816888943144"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -1026,7 +1049,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="252">
+  <cellXfs count="256">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1619,22 +1642,22 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="52" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1681,19 +1704,19 @@
     <xf numFmtId="0" fontId="21" fillId="2" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="22" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="22" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="22" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="23" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="23" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="23" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1715,6 +1738,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="5" fillId="0" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="22" fillId="10" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="22" fillId="10" borderId="36" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="24" fillId="10" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="57" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1734,7 +1766,10 @@
     <xf numFmtId="165" fontId="12" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="5" borderId="62" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -4228,11 +4263,11 @@
         </is>
       </c>
       <c r="C31" s="193" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="D31" s="194" t="n"/>
       <c r="E31" s="194" t="n">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="F31" s="194" t="n"/>
       <c r="G31" s="194" t="n"/>
@@ -4343,9 +4378,13 @@
           <t>TERMINAL</t>
         </is>
       </c>
-      <c r="C32" s="201" t="n"/>
+      <c r="C32" s="201" t="n">
+        <v>6</v>
+      </c>
       <c r="D32" s="202" t="n"/>
-      <c r="E32" s="202" t="n"/>
+      <c r="E32" s="202" t="n">
+        <v>2</v>
+      </c>
       <c r="F32" s="202" t="n"/>
       <c r="G32" s="202" t="n"/>
       <c r="H32" s="202" t="n"/>
@@ -4455,7 +4494,9 @@
           <t>ICD</t>
         </is>
       </c>
-      <c r="C33" s="201" t="n"/>
+      <c r="C33" s="201" t="n">
+        <v>1</v>
+      </c>
       <c r="D33" s="202" t="n"/>
       <c r="E33" s="202" t="n"/>
       <c r="F33" s="202" t="n"/>
@@ -4680,11 +4721,11 @@
         </is>
       </c>
       <c r="C35" s="228" t="n">
-        <v>53</v>
+        <v>198</v>
       </c>
       <c r="D35" s="210" t="n"/>
       <c r="E35" s="210" t="n">
-        <v>14</v>
+        <v>80</v>
       </c>
       <c r="F35" s="210" t="n"/>
       <c r="G35" s="210" t="n"/>
@@ -4739,15 +4780,15 @@
         </is>
       </c>
       <c r="X35" s="228" t="n">
-        <v>24</v>
+        <v>68</v>
       </c>
       <c r="Y35" s="210" t="n"/>
       <c r="Z35" s="210" t="n">
-        <v>8</v>
+        <v>80</v>
       </c>
       <c r="AA35" s="210" t="n"/>
       <c r="AB35" s="210" t="n">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="AC35" s="210" t="n"/>
       <c r="AD35" s="210" t="n"/>
@@ -4802,15 +4843,17 @@
         </is>
       </c>
       <c r="C36" s="228" t="n">
-        <v>28</v>
+        <v>205</v>
       </c>
       <c r="D36" s="210" t="n"/>
       <c r="E36" s="210" t="n">
-        <v>7</v>
-      </c>
-      <c r="F36" s="210" t="n"/>
+        <v>131</v>
+      </c>
+      <c r="F36" s="210" t="n">
+        <v>8</v>
+      </c>
       <c r="G36" s="210" t="n">
-        <v>13</v>
+        <v>42</v>
       </c>
       <c r="H36" s="210" t="n"/>
       <c r="I36" s="210" t="n"/>
@@ -4863,11 +4906,11 @@
         </is>
       </c>
       <c r="X36" s="228" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Y36" s="210" t="n"/>
       <c r="Z36" s="210" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AA36" s="210" t="n"/>
       <c r="AB36" s="210" t="n"/>
@@ -4971,11 +5014,11 @@
         </is>
       </c>
       <c r="X37" s="228" t="n">
-        <v>31</v>
+        <v>220</v>
       </c>
       <c r="Y37" s="210" t="n"/>
       <c r="Z37" s="210" t="n">
-        <v>31</v>
+        <v>199</v>
       </c>
       <c r="AA37" s="210" t="n"/>
       <c r="AB37" s="210" t="n"/>
@@ -5753,16 +5796,20 @@
           <t>TERMINAL</t>
         </is>
       </c>
-      <c r="C45" s="193" t="n"/>
+      <c r="C45" s="193" t="n">
+        <v>11</v>
+      </c>
       <c r="D45" s="194" t="n"/>
-      <c r="E45" s="194" t="n"/>
+      <c r="E45" s="194" t="n">
+        <v>20</v>
+      </c>
       <c r="F45" s="194" t="n"/>
       <c r="G45" s="194" t="n"/>
       <c r="H45" s="194" t="n"/>
       <c r="I45" s="194" t="n"/>
       <c r="J45" s="194" t="n"/>
       <c r="K45" s="195" t="n"/>
-      <c r="L45" s="216">
+      <c r="L45" s="240">
         <f>SUM(L31-C45)</f>
         <v/>
       </c>
@@ -5770,7 +5817,7 @@
         <f>SUM(M31-D45)</f>
         <v/>
       </c>
-      <c r="N45" s="217">
+      <c r="N45" s="241">
         <f>SUM(N31-E45)</f>
         <v/>
       </c>
@@ -5867,7 +5914,9 @@
       </c>
       <c r="C46" s="201" t="n"/>
       <c r="D46" s="202" t="n"/>
-      <c r="E46" s="202" t="n"/>
+      <c r="E46" s="202" t="n">
+        <v>1</v>
+      </c>
       <c r="F46" s="202" t="n"/>
       <c r="G46" s="202" t="n"/>
       <c r="H46" s="202" t="n"/>
@@ -6201,9 +6250,13 @@
           <t>DEPOT</t>
         </is>
       </c>
-      <c r="C49" s="228" t="n"/>
+      <c r="C49" s="228" t="n">
+        <v>89</v>
+      </c>
       <c r="D49" s="210" t="n"/>
-      <c r="E49" s="210" t="n"/>
+      <c r="E49" s="210" t="n">
+        <v>52</v>
+      </c>
       <c r="F49" s="210" t="n"/>
       <c r="G49" s="210" t="n"/>
       <c r="H49" s="210" t="n"/>
@@ -6256,11 +6309,19 @@
           <t>DEPOT</t>
         </is>
       </c>
-      <c r="X49" s="228" t="n"/>
+      <c r="X49" s="228" t="n">
+        <v>80</v>
+      </c>
       <c r="Y49" s="210" t="n"/>
-      <c r="Z49" s="210" t="n"/>
-      <c r="AA49" s="210" t="n"/>
-      <c r="AB49" s="210" t="n"/>
+      <c r="Z49" s="210" t="n">
+        <v>72</v>
+      </c>
+      <c r="AA49" s="210" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB49" s="210" t="n">
+        <v>8</v>
+      </c>
       <c r="AC49" s="210" t="n"/>
       <c r="AD49" s="210" t="n"/>
       <c r="AE49" s="210" t="n"/>
@@ -6313,11 +6374,19 @@
           <t>DEPOT</t>
         </is>
       </c>
-      <c r="C50" s="228" t="n"/>
+      <c r="C50" s="228" t="n">
+        <v>127</v>
+      </c>
       <c r="D50" s="210" t="n"/>
-      <c r="E50" s="210" t="n"/>
-      <c r="F50" s="210" t="n"/>
-      <c r="G50" s="210" t="n"/>
+      <c r="E50" s="210" t="n">
+        <v>127</v>
+      </c>
+      <c r="F50" s="210" t="n">
+        <v>6</v>
+      </c>
+      <c r="G50" s="210" t="n">
+        <v>24</v>
+      </c>
       <c r="H50" s="210" t="n"/>
       <c r="I50" s="210" t="n"/>
       <c r="J50" s="210" t="n"/>
@@ -6338,7 +6407,7 @@
         <f>SUM(O36-F50)</f>
         <v/>
       </c>
-      <c r="P50" s="231">
+      <c r="P50" s="242">
         <f>SUM(P36-G50)</f>
         <v/>
       </c>
@@ -6368,9 +6437,13 @@
           <t>DEPOT</t>
         </is>
       </c>
-      <c r="X50" s="228" t="n"/>
+      <c r="X50" s="228" t="n">
+        <v>11</v>
+      </c>
       <c r="Y50" s="210" t="n"/>
-      <c r="Z50" s="210" t="n"/>
+      <c r="Z50" s="210" t="n">
+        <v>11</v>
+      </c>
       <c r="AA50" s="210" t="n"/>
       <c r="AB50" s="210" t="n"/>
       <c r="AC50" s="210" t="n"/>
@@ -6472,9 +6545,13 @@
           <t>DEPOT</t>
         </is>
       </c>
-      <c r="X51" s="228" t="n"/>
+      <c r="X51" s="228" t="n">
+        <v>185</v>
+      </c>
       <c r="Y51" s="210" t="n"/>
-      <c r="Z51" s="210" t="n"/>
+      <c r="Z51" s="210" t="n">
+        <v>126</v>
+      </c>
       <c r="AA51" s="210" t="n"/>
       <c r="AB51" s="210" t="n"/>
       <c r="AC51" s="210" t="n"/>
@@ -7163,18 +7240,18 @@
           <t>HAL (THBKK)</t>
         </is>
       </c>
-      <c r="B1" s="240" t="n"/>
-      <c r="C1" s="240" t="n"/>
-      <c r="D1" s="241" t="n"/>
+      <c r="B1" s="243" t="n"/>
+      <c r="C1" s="243" t="n"/>
+      <c r="D1" s="244" t="n"/>
       <c r="E1" s="116" t="n"/>
       <c r="F1" s="172" t="inlineStr">
         <is>
           <t>HAL (THLCH)</t>
         </is>
       </c>
-      <c r="G1" s="240" t="n"/>
-      <c r="H1" s="240" t="n"/>
-      <c r="I1" s="241" t="n"/>
+      <c r="G1" s="243" t="n"/>
+      <c r="H1" s="243" t="n"/>
+      <c r="I1" s="244" t="n"/>
       <c r="J1" s="117" t="n"/>
       <c r="K1" s="117" t="n"/>
       <c r="L1" s="117" t="n"/>
@@ -7230,7 +7307,7 @@
       <c r="M2" s="117" t="n"/>
     </row>
     <row r="3" ht="16.15" customHeight="1">
-      <c r="A3" s="242" t="n"/>
+      <c r="A3" s="245" t="n"/>
       <c r="B3" s="175" t="inlineStr">
         <is>
           <t>45RE</t>
@@ -7247,7 +7324,7 @@
         </is>
       </c>
       <c r="E3" s="118" t="n"/>
-      <c r="F3" s="242" t="n"/>
+      <c r="F3" s="245" t="n"/>
       <c r="G3" s="175" t="inlineStr">
         <is>
           <t>45RE</t>
@@ -7421,20 +7498,20 @@
   </cols>
   <sheetData>
     <row r="1" ht="15.6" customHeight="1" thickBot="1">
-      <c r="B1" s="243" t="inlineStr">
+      <c r="B1" s="246" t="inlineStr">
         <is>
           <t>HAL (THBKK)</t>
         </is>
       </c>
-      <c r="C1" s="244" t="n"/>
-      <c r="D1" s="244" t="n"/>
-      <c r="E1" s="244" t="n"/>
-      <c r="F1" s="244" t="n"/>
-      <c r="G1" s="244" t="n"/>
-      <c r="H1" s="244" t="n"/>
-      <c r="I1" s="244" t="n"/>
-      <c r="J1" s="244" t="n"/>
-      <c r="K1" s="245" t="n"/>
+      <c r="C1" s="247" t="n"/>
+      <c r="D1" s="247" t="n"/>
+      <c r="E1" s="247" t="n"/>
+      <c r="F1" s="247" t="n"/>
+      <c r="G1" s="247" t="n"/>
+      <c r="H1" s="247" t="n"/>
+      <c r="I1" s="247" t="n"/>
+      <c r="J1" s="247" t="n"/>
+      <c r="K1" s="248" t="n"/>
     </row>
     <row r="2" ht="15.6" customHeight="1" thickBot="1">
       <c r="B2" s="97" t="inlineStr">
@@ -7537,39 +7614,39 @@
           <t>E/P In (this week)</t>
         </is>
       </c>
-      <c r="C4" s="246">
+      <c r="C4" s="249">
         <f>Daily!L14</f>
         <v/>
       </c>
-      <c r="D4" s="246">
+      <c r="D4" s="249">
         <f>Daily!M14</f>
         <v/>
       </c>
-      <c r="E4" s="246">
+      <c r="E4" s="249">
         <f>Daily!N14</f>
         <v/>
       </c>
-      <c r="F4" s="246">
+      <c r="F4" s="249">
         <f>Daily!O14</f>
         <v/>
       </c>
-      <c r="G4" s="246">
+      <c r="G4" s="249">
         <f>Daily!P14</f>
         <v/>
       </c>
-      <c r="H4" s="246">
+      <c r="H4" s="249">
         <f>Daily!Q14</f>
         <v/>
       </c>
-      <c r="I4" s="246">
+      <c r="I4" s="249">
         <f>Daily!R14</f>
         <v/>
       </c>
-      <c r="J4" s="246">
+      <c r="J4" s="249">
         <f>Daily!S14</f>
         <v/>
       </c>
-      <c r="K4" s="246">
+      <c r="K4" s="249">
         <f>Daily!T14</f>
         <v/>
       </c>
@@ -7604,39 +7681,39 @@
           <t>INBOUND MT RETURN</t>
         </is>
       </c>
-      <c r="C7" s="247">
+      <c r="C7" s="250">
         <f>Daily!C15</f>
         <v/>
       </c>
-      <c r="D7" s="247">
+      <c r="D7" s="250">
         <f>Daily!D15</f>
         <v/>
       </c>
-      <c r="E7" s="247">
+      <c r="E7" s="250">
         <f>Daily!E15</f>
         <v/>
       </c>
-      <c r="F7" s="247">
+      <c r="F7" s="250">
         <f>Daily!F15</f>
         <v/>
       </c>
-      <c r="G7" s="247">
+      <c r="G7" s="250">
         <f>Daily!G15</f>
         <v/>
       </c>
-      <c r="H7" s="247">
+      <c r="H7" s="250">
         <f>Daily!H15</f>
         <v/>
       </c>
-      <c r="I7" s="247">
+      <c r="I7" s="250">
         <f>Daily!I15</f>
         <v/>
       </c>
-      <c r="J7" s="247">
+      <c r="J7" s="250">
         <f>Daily!J15</f>
         <v/>
       </c>
-      <c r="K7" s="247">
+      <c r="K7" s="250">
         <f>Daily!K15</f>
         <v/>
       </c>
@@ -7647,39 +7724,39 @@
           <t>Booking(This week)</t>
         </is>
       </c>
-      <c r="C8" s="246">
+      <c r="C8" s="249">
         <f>Daily!C41</f>
         <v/>
       </c>
-      <c r="D8" s="246">
+      <c r="D8" s="249">
         <f>Daily!D41</f>
         <v/>
       </c>
-      <c r="E8" s="246">
+      <c r="E8" s="249">
         <f>Daily!E41</f>
         <v/>
       </c>
-      <c r="F8" s="246">
+      <c r="F8" s="249">
         <f>Daily!F41</f>
         <v/>
       </c>
-      <c r="G8" s="246">
+      <c r="G8" s="249">
         <f>Daily!G41</f>
         <v/>
       </c>
-      <c r="H8" s="246">
+      <c r="H8" s="249">
         <f>Daily!H41</f>
         <v/>
       </c>
-      <c r="I8" s="246">
+      <c r="I8" s="249">
         <f>Daily!I41</f>
         <v/>
       </c>
-      <c r="J8" s="246">
+      <c r="J8" s="249">
         <f>Daily!J41</f>
         <v/>
       </c>
-      <c r="K8" s="246">
+      <c r="K8" s="249">
         <f>Daily!K41</f>
         <v/>
       </c>
@@ -7694,39 +7771,39 @@
           <t>Booking(Next week)</t>
         </is>
       </c>
-      <c r="C9" s="248">
+      <c r="C9" s="251">
         <f>Daily!C55</f>
         <v/>
       </c>
-      <c r="D9" s="248">
+      <c r="D9" s="251">
         <f>Daily!D55</f>
         <v/>
       </c>
-      <c r="E9" s="248">
+      <c r="E9" s="251">
         <f>Daily!E55</f>
         <v/>
       </c>
-      <c r="F9" s="248">
+      <c r="F9" s="251">
         <f>Daily!F55</f>
         <v/>
       </c>
-      <c r="G9" s="248">
+      <c r="G9" s="251">
         <f>Daily!G55</f>
         <v/>
       </c>
-      <c r="H9" s="248">
+      <c r="H9" s="251">
         <f>Daily!H55</f>
         <v/>
       </c>
-      <c r="I9" s="248">
+      <c r="I9" s="251">
         <f>Daily!I55</f>
         <v/>
       </c>
-      <c r="J9" s="248">
+      <c r="J9" s="251">
         <f>Daily!J55</f>
         <v/>
       </c>
-      <c r="K9" s="248">
+      <c r="K9" s="251">
         <f>Daily!K55</f>
         <v/>
       </c>
@@ -7741,39 +7818,39 @@
           <t>Balance</t>
         </is>
       </c>
-      <c r="C10" s="249">
+      <c r="C10" s="252">
         <f>SUM(C3+C4+C5+C6+C7-C8-C9)</f>
         <v/>
       </c>
-      <c r="D10" s="249">
+      <c r="D10" s="252">
         <f>SUM(D3+D4+D5+D6+D7-D8-D9)</f>
         <v/>
       </c>
-      <c r="E10" s="249">
+      <c r="E10" s="252">
         <f>SUM(E3+E4+E5+E6+E7-E8-E9)</f>
         <v/>
       </c>
-      <c r="F10" s="249">
+      <c r="F10" s="252">
         <f>SUM(F3+F4+F5+F6+F7-F8-F9)</f>
         <v/>
       </c>
-      <c r="G10" s="249">
+      <c r="G10" s="253">
         <f>SUM(G3+G4+G5+G6+G7-G8-G9)</f>
         <v/>
       </c>
-      <c r="H10" s="249">
+      <c r="H10" s="252">
         <f>SUM(H3+H4+H5+H6+H7-H8-H9)</f>
         <v/>
       </c>
-      <c r="I10" s="249">
+      <c r="I10" s="252">
         <f>SUM(I3+I4+I5+I6+I7-I8-I9)</f>
         <v/>
       </c>
-      <c r="J10" s="249">
+      <c r="J10" s="252">
         <f>SUM(J3+J4+J5+J6+J7-J8-J9)</f>
         <v/>
       </c>
-      <c r="K10" s="249">
+      <c r="K10" s="252">
         <f>SUM(K3+K4+K5+K6+K7-K8-K9)</f>
         <v/>
       </c>
@@ -7791,20 +7868,20 @@
       <c r="K11" s="111" t="n"/>
     </row>
     <row r="12" ht="15.6" customHeight="1" thickBot="1">
-      <c r="B12" s="250" t="inlineStr">
+      <c r="B12" s="254" t="inlineStr">
         <is>
           <t>HAL (THLCH)</t>
         </is>
       </c>
-      <c r="C12" s="244" t="n"/>
-      <c r="D12" s="244" t="n"/>
-      <c r="E12" s="244" t="n"/>
-      <c r="F12" s="244" t="n"/>
-      <c r="G12" s="244" t="n"/>
-      <c r="H12" s="244" t="n"/>
-      <c r="I12" s="244" t="n"/>
-      <c r="J12" s="244" t="n"/>
-      <c r="K12" s="245" t="n"/>
+      <c r="C12" s="247" t="n"/>
+      <c r="D12" s="247" t="n"/>
+      <c r="E12" s="247" t="n"/>
+      <c r="F12" s="247" t="n"/>
+      <c r="G12" s="247" t="n"/>
+      <c r="H12" s="247" t="n"/>
+      <c r="I12" s="247" t="n"/>
+      <c r="J12" s="247" t="n"/>
+      <c r="K12" s="248" t="n"/>
     </row>
     <row r="13" ht="15.6" customHeight="1" thickBot="1">
       <c r="B13" s="97" t="inlineStr">
@@ -7907,39 +7984,39 @@
           <t>E/P In (this week)</t>
         </is>
       </c>
-      <c r="C15" s="246">
+      <c r="C15" s="249">
         <f>Daily!AG14</f>
         <v/>
       </c>
-      <c r="D15" s="246">
+      <c r="D15" s="249">
         <f>Daily!AH14</f>
         <v/>
       </c>
-      <c r="E15" s="246">
+      <c r="E15" s="249">
         <f>Daily!AI14</f>
         <v/>
       </c>
-      <c r="F15" s="246">
+      <c r="F15" s="249">
         <f>Daily!AJ14</f>
         <v/>
       </c>
-      <c r="G15" s="246">
+      <c r="G15" s="249">
         <f>Daily!AK14</f>
         <v/>
       </c>
-      <c r="H15" s="246">
+      <c r="H15" s="249">
         <f>Daily!AL14</f>
         <v/>
       </c>
-      <c r="I15" s="246">
+      <c r="I15" s="249">
         <f>Daily!AM14</f>
         <v/>
       </c>
-      <c r="J15" s="246">
+      <c r="J15" s="249">
         <f>Daily!AN14</f>
         <v/>
       </c>
-      <c r="K15" s="246">
+      <c r="K15" s="249">
         <f>Daily!AO14</f>
         <v/>
       </c>
@@ -7974,39 +8051,39 @@
           <t>INBOUND MT RETURN</t>
         </is>
       </c>
-      <c r="C18" s="247">
+      <c r="C18" s="250">
         <f>Daily!X15</f>
         <v/>
       </c>
-      <c r="D18" s="247">
+      <c r="D18" s="250">
         <f>Daily!Y15</f>
         <v/>
       </c>
-      <c r="E18" s="247">
+      <c r="E18" s="250">
         <f>Daily!Z15</f>
         <v/>
       </c>
-      <c r="F18" s="247">
+      <c r="F18" s="250">
         <f>Daily!AA15</f>
         <v/>
       </c>
-      <c r="G18" s="247">
+      <c r="G18" s="250">
         <f>Daily!AB15</f>
         <v/>
       </c>
-      <c r="H18" s="247">
+      <c r="H18" s="250">
         <f>Daily!AC15</f>
         <v/>
       </c>
-      <c r="I18" s="247">
+      <c r="I18" s="250">
         <f>Daily!AD15</f>
         <v/>
       </c>
-      <c r="J18" s="247">
+      <c r="J18" s="250">
         <f>Daily!AE15</f>
         <v/>
       </c>
-      <c r="K18" s="247">
+      <c r="K18" s="250">
         <f>Daily!AF15</f>
         <v/>
       </c>
@@ -8017,39 +8094,39 @@
           <t>Booking(This week)</t>
         </is>
       </c>
-      <c r="C19" s="248">
+      <c r="C19" s="251">
         <f>Daily!X41</f>
         <v/>
       </c>
-      <c r="D19" s="248">
+      <c r="D19" s="251">
         <f>Daily!Y41</f>
         <v/>
       </c>
-      <c r="E19" s="248">
+      <c r="E19" s="251">
         <f>Daily!Z41</f>
         <v/>
       </c>
-      <c r="F19" s="248">
+      <c r="F19" s="251">
         <f>Daily!AA41</f>
         <v/>
       </c>
-      <c r="G19" s="248">
+      <c r="G19" s="251">
         <f>Daily!AB41</f>
         <v/>
       </c>
-      <c r="H19" s="248">
+      <c r="H19" s="251">
         <f>Daily!AC41</f>
         <v/>
       </c>
-      <c r="I19" s="251">
+      <c r="I19" s="255">
         <f>Daily!AD41</f>
         <v/>
       </c>
-      <c r="J19" s="251">
+      <c r="J19" s="255">
         <f>Daily!AE41</f>
         <v/>
       </c>
-      <c r="K19" s="248">
+      <c r="K19" s="251">
         <f>Daily!AF41</f>
         <v/>
       </c>
@@ -8064,39 +8141,39 @@
           <t>Booking(Next week)</t>
         </is>
       </c>
-      <c r="C20" s="248">
+      <c r="C20" s="251">
         <f>Daily!X55</f>
         <v/>
       </c>
-      <c r="D20" s="248">
+      <c r="D20" s="251">
         <f>Daily!Y55</f>
         <v/>
       </c>
-      <c r="E20" s="248">
+      <c r="E20" s="251">
         <f>Daily!Z55</f>
         <v/>
       </c>
-      <c r="F20" s="248">
+      <c r="F20" s="251">
         <f>Daily!AA55</f>
         <v/>
       </c>
-      <c r="G20" s="248">
+      <c r="G20" s="251">
         <f>Daily!AB55</f>
         <v/>
       </c>
-      <c r="H20" s="248">
+      <c r="H20" s="251">
         <f>Daily!AC55</f>
         <v/>
       </c>
-      <c r="I20" s="248">
+      <c r="I20" s="251">
         <f>Daily!AD55</f>
         <v/>
       </c>
-      <c r="J20" s="248">
+      <c r="J20" s="251">
         <f>Daily!AE55</f>
         <v/>
       </c>
-      <c r="K20" s="248">
+      <c r="K20" s="251">
         <f>Daily!AF55</f>
         <v/>
       </c>
@@ -8111,39 +8188,39 @@
           <t>Balance</t>
         </is>
       </c>
-      <c r="C21" s="249">
+      <c r="C21" s="252">
         <f>SUM(C14+C15+C16+C17+C18-C19-C20)</f>
         <v/>
       </c>
-      <c r="D21" s="249">
+      <c r="D21" s="252">
         <f>SUM(D14+D15+D16+D17+D18-D19-D20)</f>
         <v/>
       </c>
-      <c r="E21" s="249">
+      <c r="E21" s="252">
         <f>SUM(E14+E15+E16+E17+E18-E19-E20)</f>
         <v/>
       </c>
-      <c r="F21" s="249">
+      <c r="F21" s="252">
         <f>SUM(F14+F15+F16+F17+F18-F19-F20)</f>
         <v/>
       </c>
-      <c r="G21" s="249">
+      <c r="G21" s="252">
         <f>SUM(G14+G15+G16+G17+G18-G19-G20)</f>
         <v/>
       </c>
-      <c r="H21" s="249">
+      <c r="H21" s="252">
         <f>SUM(H14+H15+H16+H17+H18-H19-H20)</f>
         <v/>
       </c>
-      <c r="I21" s="249">
+      <c r="I21" s="252">
         <f>SUM(I14+I15+I16+I17+I18-I19-I20)</f>
         <v/>
       </c>
-      <c r="J21" s="249">
+      <c r="J21" s="252">
         <f>SUM(J14+J15+J16+J17+J18-J19-J20)</f>
         <v/>
       </c>
-      <c r="K21" s="249">
+      <c r="K21" s="252">
         <f>SUM(K14+K15+K16+K17+K18-K19-K20)</f>
         <v/>
       </c>

</xml_diff>